<commit_message>
Large update to both regression and probability models
Updated all models and underlying data to include 2025, including some code fixes to ensure smooth model runs from FPL API, and create defensive contribution calculation
</commit_message>
<xml_diff>
--- a/Probability model/data/Probability model peformance.xlsx
+++ b/Probability model/data/Probability model peformance.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t xml:space="preserve">stat</t>
   </si>
@@ -36,6 +36,9 @@
     <t xml:space="preserve">cs_points</t>
   </si>
   <si>
+    <t xml:space="preserve">defense_points</t>
+  </si>
+  <si>
     <t xml:space="preserve">goal_points</t>
   </si>
   <si>
@@ -48,6 +51,9 @@
     <t xml:space="preserve">pen_saves_points</t>
   </si>
   <si>
+    <t xml:space="preserve">points_per_week</t>
+  </si>
+  <si>
     <t xml:space="preserve">save_points</t>
   </si>
   <si>
@@ -66,10 +72,10 @@
     <t xml:space="preserve">Actual_position_rank - expected_position_rank</t>
   </si>
   <si>
+    <t xml:space="preserve">GKP</t>
+  </si>
+  <si>
     <t xml:space="preserve">DEF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GKP</t>
   </si>
   <si>
     <t xml:space="preserve">MID</t>
@@ -420,10 +426,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="n">
-        <v>1.72972972972973</v>
+        <v>0.6128</v>
       </c>
       <c r="C2" t="n">
-        <v>-3.89527027027027</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -431,10 +437,10 @@
         <v>4</v>
       </c>
       <c r="B3" t="n">
-        <v>-6.48310810810811</v>
+        <v>-3.632</v>
       </c>
       <c r="C3" t="n">
-        <v>121.030405405405</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -442,10 +448,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="n">
-        <v>1.05067567567568</v>
+        <v>1.1168</v>
       </c>
       <c r="C4" t="n">
-        <v>7.55405405405405</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -453,10 +459,10 @@
         <v>6</v>
       </c>
       <c r="B5" t="n">
-        <v>3.57432432432432</v>
+        <v>4.656</v>
       </c>
       <c r="C5" t="n">
-        <v>-1.81081081081081</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -464,10 +470,10 @@
         <v>7</v>
       </c>
       <c r="B6" t="n">
-        <v>2.05743243243243</v>
+        <v>-0.1904</v>
       </c>
       <c r="C6" t="n">
-        <v>27.75</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -475,10 +481,10 @@
         <v>8</v>
       </c>
       <c r="B7" t="n">
-        <v>-3.14527027027027</v>
+        <v>-0.4336</v>
       </c>
       <c r="C7" t="n">
-        <v>156.902027027027</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -486,10 +492,10 @@
         <v>9</v>
       </c>
       <c r="B8" t="n">
-        <v>-0.195945945945946</v>
+        <v>-0.9152</v>
       </c>
       <c r="C8" t="n">
-        <v>6.49324324324324</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -497,10 +503,10 @@
         <v>10</v>
       </c>
       <c r="B9" t="n">
-        <v>0.0709459459459459</v>
+        <v>-0.1248</v>
       </c>
       <c r="C9" t="n">
-        <v>-1.58108108108108</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -508,10 +514,10 @@
         <v>11</v>
       </c>
       <c r="B10" t="n">
-        <v>1.45945945945946</v>
+        <v>0.0384</v>
       </c>
       <c r="C10" t="n">
-        <v>-6.83445945945946</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -519,10 +525,10 @@
         <v>12</v>
       </c>
       <c r="B11" t="n">
-        <v>-0.790540540540541</v>
+        <v>-1.10224138752311</v>
       </c>
       <c r="C11" t="n">
-        <v>5.6722972972973</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -530,10 +536,10 @@
         <v>13</v>
       </c>
       <c r="B12" t="n">
-        <v>-42.6486486486486</v>
+        <v>0.7168</v>
       </c>
       <c r="C12" t="n">
-        <v>166.672297297297</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -541,10 +547,32 @@
         <v>14</v>
       </c>
       <c r="B13" t="n">
-        <v>20.2364864864865</v>
+        <v>-0.9968</v>
       </c>
       <c r="C13" t="n">
-        <v>-4.00337837837838</v>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14" t="n">
+        <v>-26.5472</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" t="n">
+        <v>12.8752</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -560,7 +588,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -569,222 +597,222 @@
         <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
       </c>
       <c r="C2" t="n">
-        <v>0.862385321100917</v>
+        <v>0.25</v>
       </c>
       <c r="D2" t="n">
-        <v>2.44954128440367</v>
+        <v>2.58333333333333</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B3" t="s">
         <v>3</v>
       </c>
       <c r="C3" t="n">
-        <v>0.681818181818182</v>
+        <v>1.26890756302521</v>
       </c>
       <c r="D3" t="n">
-        <v>0.636363636363636</v>
+        <v>5.42857142857143</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B4" t="s">
         <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>2.71532846715328</v>
+        <v>2.01418439716312</v>
       </c>
       <c r="D4" t="n">
-        <v>-3.8029197080292</v>
+        <v>-3.17021276595745</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B5" t="s">
         <v>3</v>
       </c>
       <c r="C5" t="n">
-        <v>1.10714285714286</v>
+        <v>1.32258064516129</v>
       </c>
       <c r="D5" t="n">
-        <v>-2.03571428571429</v>
+        <v>-2.48387096774194</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B6" t="s">
         <v>4</v>
       </c>
       <c r="C6" t="n">
-        <v>-4.58715596330275</v>
+        <v>-6.45833333333333</v>
       </c>
       <c r="D6" t="n">
-        <v>41.8440366972477</v>
+        <v>25.125</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B7" t="s">
         <v>4</v>
       </c>
       <c r="C7" t="n">
-        <v>-7.68181818181818</v>
+        <v>-4.52100840336134</v>
       </c>
       <c r="D7" t="n">
-        <v>26.6818181818182</v>
+        <v>35.9747899159664</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B8" t="s">
         <v>4</v>
       </c>
       <c r="C8" t="n">
-        <v>-6.24087591240876</v>
+        <v>-6.17021276595745</v>
       </c>
       <c r="D8" t="n">
-        <v>40.9051094890511</v>
+        <v>54.7234042553191</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B9" t="s">
         <v>4</v>
       </c>
       <c r="C9" t="n">
-        <v>-14.1071428571429</v>
+        <v>-11.6129032258065</v>
       </c>
       <c r="D9" t="n">
-        <v>17.6071428571429</v>
+        <v>13.6774193548387</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B10" t="s">
         <v>5</v>
       </c>
       <c r="C10" t="n">
-        <v>1.22018348623853</v>
+        <v>0.958333333333333</v>
       </c>
       <c r="D10" t="n">
-        <v>3.00917431192661</v>
+        <v>-2.75</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B11" t="s">
         <v>5</v>
       </c>
       <c r="C11" t="n">
-        <v>0.545454545454545</v>
+        <v>1.2436974789916</v>
       </c>
       <c r="D11" t="n">
-        <v>-3.54545454545455</v>
+        <v>0.915966386554622</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B12" t="s">
         <v>5</v>
       </c>
       <c r="C12" t="n">
-        <v>1.07299270072993</v>
+        <v>1.34042553191489</v>
       </c>
       <c r="D12" t="n">
-        <v>2.86131386861314</v>
+        <v>2.63120567375887</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B13" t="s">
         <v>5</v>
       </c>
       <c r="C13" t="n">
-        <v>0.678571428571429</v>
+        <v>1.06451612903226</v>
       </c>
       <c r="D13" t="n">
-        <v>2.32142857142857</v>
+        <v>1.54838709677419</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B14" t="s">
         <v>6</v>
       </c>
       <c r="C14" t="n">
-        <v>5.3302752293578</v>
+        <v>16.75</v>
       </c>
       <c r="D14" t="n">
-        <v>1.71559633027523</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B15" t="s">
         <v>6</v>
       </c>
       <c r="C15" t="n">
-        <v>5.31818181818182</v>
+        <v>14.8319327731092</v>
       </c>
       <c r="D15" t="n">
-        <v>2.22727272727273</v>
+        <v>1.28571428571429</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B16" t="s">
         <v>6</v>
       </c>
       <c r="C16" t="n">
-        <v>2.62773722627737</v>
+        <v>4.26241134751773</v>
       </c>
       <c r="D16" t="n">
-        <v>-1.48905109489051</v>
+        <v>-7.32624113475177</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B17" t="s">
         <v>6</v>
@@ -798,259 +826,259 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B18" t="s">
         <v>7</v>
       </c>
       <c r="C18" t="n">
-        <v>-0.532110091743119</v>
+        <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>22.9082568807339</v>
+        <v>-2.75</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B19" t="s">
         <v>7</v>
       </c>
       <c r="C19" t="n">
-        <v>-1.13636363636364</v>
+        <v>0</v>
       </c>
       <c r="D19" t="n">
-        <v>5.63636363636364</v>
+        <v>-2.63865546218487</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B20" t="s">
         <v>7</v>
       </c>
       <c r="C20" t="n">
-        <v>3.33576642335766</v>
+        <v>0</v>
       </c>
       <c r="D20" t="n">
-        <v>4.43065693430657</v>
+        <v>-1.43971631205674</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B21" t="s">
         <v>7</v>
       </c>
       <c r="C21" t="n">
-        <v>8.39285714285714</v>
+        <v>0</v>
       </c>
       <c r="D21" t="n">
-        <v>-0.892857142857143</v>
+        <v>-0.193548387096774</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B22" t="s">
         <v>8</v>
       </c>
       <c r="C22" t="n">
-        <v>3.03669724770642</v>
+        <v>-0.958333333333333</v>
       </c>
       <c r="D22" t="n">
-        <v>46.3119266055046</v>
+        <v>-1.41666666666667</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B23" t="s">
         <v>8</v>
       </c>
       <c r="C23" t="n">
-        <v>1.09090909090909</v>
+        <v>-0.588235294117647</v>
       </c>
       <c r="D23" t="n">
-        <v>23.9090909090909</v>
+        <v>12.546218487395</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B24" t="s">
         <v>8</v>
       </c>
       <c r="C24" t="n">
-        <v>-7.64963503649635</v>
+        <v>2.19858156028369</v>
       </c>
       <c r="D24" t="n">
-        <v>60.3649635036496</v>
+        <v>-3.02127659574468</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B25" t="s">
         <v>8</v>
       </c>
       <c r="C25" t="n">
-        <v>-8.5</v>
+        <v>7.16129032258065</v>
       </c>
       <c r="D25" t="n">
-        <v>15.5</v>
+        <v>-3.2258064516129</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B26" t="s">
         <v>9</v>
       </c>
       <c r="C26" t="n">
-        <v>-0.293577981651376</v>
+        <v>-3</v>
       </c>
       <c r="D26" t="n">
-        <v>2.39449541284404</v>
+        <v>24.3333333333333</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B27" t="s">
         <v>9</v>
       </c>
       <c r="C27" t="n">
-        <v>0</v>
+        <v>-1.01680672268908</v>
       </c>
       <c r="D27" t="n">
-        <v>0.136363636363636</v>
+        <v>42.9075630252101</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B28" t="s">
         <v>9</v>
       </c>
       <c r="C28" t="n">
-        <v>-0.160583941605839</v>
+        <v>-6.05673758865248</v>
       </c>
       <c r="D28" t="n">
-        <v>3.1970802919708</v>
+        <v>48.4822695035461</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B29" t="s">
         <v>9</v>
       </c>
       <c r="C29" t="n">
-        <v>-0.142857142857143</v>
+        <v>-5.48387096774194</v>
       </c>
       <c r="D29" t="n">
-        <v>-0.321428571428571</v>
+        <v>18.4193548387097</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B30" t="s">
         <v>10</v>
       </c>
       <c r="C30" t="n">
-        <v>0</v>
+        <v>-0.208333333333333</v>
       </c>
       <c r="D30" t="n">
-        <v>0</v>
+        <v>0.0833333333333333</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B31" t="s">
         <v>10</v>
       </c>
       <c r="C31" t="n">
-        <v>0.954545454545455</v>
+        <v>-0.34453781512605</v>
       </c>
       <c r="D31" t="n">
-        <v>2.22727272727273</v>
+        <v>3.61344537815126</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B32" t="s">
         <v>10</v>
       </c>
       <c r="C32" t="n">
-        <v>0</v>
+        <v>-0.134751773049645</v>
       </c>
       <c r="D32" t="n">
-        <v>0</v>
+        <v>1.71631205673759</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B33" t="s">
         <v>10</v>
       </c>
       <c r="C33" t="n">
-        <v>0</v>
+        <v>-0.225806451612903</v>
       </c>
       <c r="D33" t="n">
-        <v>0</v>
+        <v>-2.35483870967742</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B34" t="s">
         <v>11</v>
       </c>
       <c r="C34" t="n">
-        <v>0</v>
+        <v>0.958333333333333</v>
       </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>-1.375</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B35" t="s">
         <v>11</v>
       </c>
       <c r="C35" t="n">
-        <v>19.6363636363636</v>
+        <v>0</v>
       </c>
       <c r="D35" t="n">
-        <v>-29.3181818181818</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B36" t="s">
         <v>11</v>
@@ -1064,7 +1092,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B37" t="s">
         <v>11</v>
@@ -1078,170 +1106,282 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B38" t="s">
         <v>12</v>
       </c>
       <c r="C38" t="n">
-        <v>0</v>
+        <v>-2.36516659282146</v>
       </c>
       <c r="D38" t="n">
-        <v>0</v>
+        <v>26.5416666666667</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B39" t="s">
         <v>12</v>
       </c>
       <c r="C39" t="n">
-        <v>-10.6363636363636</v>
+        <v>-1.56132218490425</v>
       </c>
       <c r="D39" t="n">
-        <v>28.6818181818182</v>
+        <v>47.6806722689076</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B40" t="s">
         <v>12</v>
       </c>
       <c r="C40" t="n">
-        <v>0</v>
+        <v>-1.92637912828891</v>
       </c>
       <c r="D40" t="n">
-        <v>0</v>
+        <v>65.5744680851064</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B41" t="s">
         <v>12</v>
       </c>
       <c r="C41" t="n">
-        <v>0</v>
+        <v>-2.32804475045785</v>
       </c>
       <c r="D41" t="n">
-        <v>0</v>
+        <v>15.2258064516129</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B42" t="s">
         <v>13</v>
       </c>
       <c r="C42" t="n">
-        <v>-41.2752293577982</v>
+        <v>17.3333333333333</v>
       </c>
       <c r="D42" t="n">
-        <v>59.7798165137615</v>
+        <v>-26.7916666666667</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B43" t="s">
         <v>13</v>
       </c>
       <c r="C43" t="n">
-        <v>-48.7272727272727</v>
+        <v>0</v>
       </c>
       <c r="D43" t="n">
-        <v>29.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B44" t="s">
         <v>13</v>
       </c>
       <c r="C44" t="n">
-        <v>-42.4233576642336</v>
+        <v>0</v>
       </c>
       <c r="D44" t="n">
-        <v>59.5328467153285</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B45" t="s">
         <v>13</v>
       </c>
       <c r="C45" t="n">
-        <v>-44.3214285714286</v>
+        <v>0</v>
       </c>
       <c r="D45" t="n">
-        <v>19.6785714285714</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B46" t="s">
         <v>14</v>
       </c>
       <c r="C46" t="n">
-        <v>17.1743119266055</v>
+        <v>-22.9166666666667</v>
       </c>
       <c r="D46" t="n">
-        <v>0.293577981651376</v>
+        <v>26.625</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B47" t="s">
         <v>14</v>
       </c>
       <c r="C47" t="n">
-        <v>23.0909090909091</v>
+        <v>0</v>
       </c>
       <c r="D47" t="n">
-        <v>0.0454545454545455</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B48" t="s">
         <v>14</v>
       </c>
       <c r="C48" t="n">
-        <v>21.0875912408759</v>
+        <v>0</v>
       </c>
       <c r="D48" t="n">
-        <v>-1.46715328467153</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B49" t="s">
         <v>14</v>
       </c>
       <c r="C49" t="n">
-        <v>25.75</v>
+        <v>0</v>
       </c>
       <c r="D49" t="n">
-        <v>-0.285714285714286</v>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="s">
+        <v>19</v>
+      </c>
+      <c r="B50" t="s">
+        <v>15</v>
+      </c>
+      <c r="C50" t="n">
+        <v>-50.625</v>
+      </c>
+      <c r="D50" t="n">
+        <v>26.7916666666667</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="s">
+        <v>20</v>
+      </c>
+      <c r="B51" t="s">
+        <v>15</v>
+      </c>
+      <c r="C51" t="n">
+        <v>-43.5378151260504</v>
+      </c>
+      <c r="D51" t="n">
+        <v>48.2268907563025</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="s">
+        <v>21</v>
+      </c>
+      <c r="B52" t="s">
+        <v>15</v>
+      </c>
+      <c r="C52" t="n">
+        <v>-43.936170212766</v>
+      </c>
+      <c r="D52" t="n">
+        <v>67.2836879432624</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="s">
+        <v>22</v>
+      </c>
+      <c r="B53" t="s">
+        <v>15</v>
+      </c>
+      <c r="C53" t="n">
+        <v>-41.0645161290323</v>
+      </c>
+      <c r="D53" t="n">
+        <v>16.0322580645161</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="s">
+        <v>19</v>
+      </c>
+      <c r="B54" t="s">
+        <v>16</v>
+      </c>
+      <c r="C54" t="n">
+        <v>11.4166666666667</v>
+      </c>
+      <c r="D54" t="n">
+        <v>-0.291666666666667</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="s">
+        <v>20</v>
+      </c>
+      <c r="B55" t="s">
+        <v>16</v>
+      </c>
+      <c r="C55" t="n">
+        <v>32.9075630252101</v>
+      </c>
+      <c r="D55" t="n">
+        <v>-1.57142857142857</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="s">
+        <v>21</v>
+      </c>
+      <c r="B56" t="s">
+        <v>16</v>
+      </c>
+      <c r="C56" t="n">
+        <v>23.9645390070922</v>
+      </c>
+      <c r="D56" t="n">
+        <v>-5.57446808510638</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="s">
+        <v>22</v>
+      </c>
+      <c r="B57" t="s">
+        <v>16</v>
+      </c>
+      <c r="C57" t="n">
+        <v>22.7741935483871</v>
+      </c>
+      <c r="D57" t="n">
+        <v>-3.29032258064516</v>
       </c>
     </row>
   </sheetData>

</xml_diff>